<commit_message>
Think I'm done with Lab8
</commit_message>
<xml_diff>
--- a/Lab B/Lab8/L8E2.xlsx
+++ b/Lab B/Lab8/L8E2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teva\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\School\openu-courses\Lab B\Lab8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2346D33-9A74-40BF-BDE6-5FFBEFBD07C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10355E42-21CE-4B1E-A27C-F595FBACC0D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{AE432DE3-28B7-4759-BADC-E87FFEFAB150}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{AE432DE3-28B7-4759-BADC-E87FFEFAB150}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,16 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -53,7 +61,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
@@ -101,7 +109,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="he-IL"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -113,6 +121,36 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="he-IL"/>
+              <a:t>מתח</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="he-IL" baseline="0"/>
+              <a:t> רכיבים כפונקציה של תדירות</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -149,133 +187,11 @@
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="1"/>
           <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>גיליון1!$B$3:$B$27</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
-                <c:pt idx="0">
-                  <c:v>5.48</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>5.96</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>6.47</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>6.96</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>7.07</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>7.16</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>7.26</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>7.37</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>7.47</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>7.57</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>7.67</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>7.78</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>7.8840000000000003</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>7.96</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>8.07</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>8.17</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>8.26</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>8.36</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>8.4600000000000009</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>8.57</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>8.66</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>8.76</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>9.26</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>9.76</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>10.27</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>גיליון1!$C$3:$C$27</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="25"/>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-26B4-4CFC-B6B7-45B53B317EF0}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
+          <c:tx>
+            <c:v>מתח נגד</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
               <a:noFill/>
@@ -475,7 +391,10 @@
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>מתח סליל</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
               <a:noFill/>
@@ -675,7 +594,10 @@
         </c:ser>
         <c:ser>
           <c:idx val="3"/>
-          <c:order val="3"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>מתח קבל</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
               <a:noFill/>
@@ -887,7 +809,9 @@
       <c:valAx>
         <c:axId val="546492927"/>
         <c:scaling>
-          <c:orientation val="maxMin"/>
+          <c:orientation val="minMax"/>
+          <c:max val="11"/>
+          <c:min val="5"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -905,8 +829,72 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>[kHz]</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="he-IL" baseline="0"/>
+                  <a:t>תדירות</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -952,7 +940,7 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="r"/>
+        <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -967,8 +955,76 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="he-IL"/>
+                  <a:t>[</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>V</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="he-IL"/>
+                  <a:t>]</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="he-IL" baseline="0"/>
+                  <a:t> מתח</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1043,12 +1099,13 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="he-IL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1056,7 +1113,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1652,15 +1708,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:colOff>125730</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>388620</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1689,9 +1745,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1729,7 +1785,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1835,7 +1891,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1977,7 +2033,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1986,9 +2042,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90532824-3769-4444-BD96-1674CBB392EE}">
   <dimension ref="B2:F27"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -2005,10 +2061,14 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>5.48</v>
       </c>
+      <c r="C3">
+        <f>2*PI() * B3</f>
+        <v>34.431855483344137</v>
+      </c>
       <c r="D3">
         <v>0.5</v>
       </c>
@@ -2019,10 +2079,14 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>5.96</v>
       </c>
+      <c r="C4">
+        <f t="shared" ref="C4:C27" si="0">2*PI() * B4</f>
+        <v>37.447784430790335</v>
+      </c>
       <c r="D4">
         <v>0.65</v>
       </c>
@@ -2033,10 +2097,14 @@
         <v>4.95</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>6.47</v>
       </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>40.652208937451924</v>
+      </c>
       <c r="D5">
         <v>0.89</v>
       </c>
@@ -2047,10 +2115,14 @@
         <v>6.16</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>6.96</v>
       </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>43.730969737969922</v>
+      </c>
       <c r="D6">
         <v>1.24</v>
       </c>
@@ -2061,10 +2133,14 @@
         <v>7.88</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>7.07</v>
       </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>44.422120121759676</v>
+      </c>
       <c r="D7">
         <v>1.34</v>
       </c>
@@ -2075,10 +2151,14 @@
         <v>8.34</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>7.16</v>
       </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>44.987606799405839</v>
+      </c>
       <c r="D8">
         <v>1.43</v>
       </c>
@@ -2089,10 +2169,14 @@
         <v>8.74</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>7.26</v>
       </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>45.615925330123794</v>
+      </c>
       <c r="D9">
         <v>1.52</v>
       </c>
@@ -2103,10 +2187,14 @@
         <v>9.17</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>7.37</v>
       </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>46.307075713913548</v>
+      </c>
       <c r="D10">
         <v>1.61</v>
       </c>
@@ -2117,10 +2205,14 @@
         <v>9.58</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>7.47</v>
       </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>46.93539424463151</v>
+      </c>
       <c r="D11">
         <v>1.71</v>
       </c>
@@ -2131,10 +2223,14 @@
         <v>9.99</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>7.57</v>
       </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>47.563712775349472</v>
+      </c>
       <c r="D12">
         <v>1.78</v>
       </c>
@@ -2145,10 +2241,14 @@
         <v>10.25</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>7.67</v>
       </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>48.192031306067427</v>
+      </c>
       <c r="D13">
         <v>1.85</v>
       </c>
@@ -2159,10 +2259,14 @@
         <v>10.51</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14">
         <v>7.78</v>
       </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>48.883181689857182</v>
+      </c>
       <c r="D14">
         <v>1.88</v>
       </c>
@@ -2173,10 +2277,14 @@
         <v>10.58</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>7.8840000000000003</v>
       </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>49.536632961803861</v>
+      </c>
       <c r="D15">
         <v>1.89</v>
       </c>
@@ -2187,10 +2295,14 @@
         <v>10.51</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16">
         <v>7.96</v>
       </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>50.014155045149508</v>
+      </c>
       <c r="D16">
         <v>1.89</v>
       </c>
@@ -2201,10 +2313,14 @@
         <v>10.38</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>8.07</v>
       </c>
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>50.705305428939262</v>
+      </c>
       <c r="D17">
         <v>1.84</v>
       </c>
@@ -2215,10 +2331,14 @@
         <v>10.02</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>8.17</v>
       </c>
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>51.333623959657217</v>
+      </c>
       <c r="D18">
         <v>1.79</v>
       </c>
@@ -2229,10 +2349,14 @@
         <v>9.6199999999999992</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>8.26</v>
       </c>
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>51.89911063730338</v>
+      </c>
       <c r="D19">
         <v>1.73</v>
       </c>
@@ -2243,10 +2367,14 @@
         <v>9.24</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>8.36</v>
       </c>
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>52.527429168021335</v>
+      </c>
       <c r="D20">
         <v>1.65</v>
       </c>
@@ -2257,10 +2385,14 @@
         <v>8.74</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>8.4600000000000009</v>
       </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>53.155747698739304</v>
+      </c>
       <c r="D21">
         <v>1.58</v>
       </c>
@@ -2271,10 +2403,14 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>8.57</v>
       </c>
+      <c r="C22">
+        <f t="shared" si="0"/>
+        <v>53.846898082529059</v>
+      </c>
       <c r="D22">
         <v>1.49</v>
       </c>
@@ -2285,10 +2421,14 @@
         <v>7.72</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>8.66</v>
       </c>
+      <c r="C23">
+        <f t="shared" si="0"/>
+        <v>54.412384760175215</v>
+      </c>
       <c r="D23">
         <v>1.41</v>
       </c>
@@ -2299,10 +2439,14 @@
         <v>7.29</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24">
         <v>8.76</v>
       </c>
+      <c r="C24">
+        <f t="shared" si="0"/>
+        <v>55.040703290893177</v>
+      </c>
       <c r="D24">
         <v>1.33</v>
       </c>
@@ -2313,10 +2457,14 @@
         <v>6.83</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25">
         <v>9.26</v>
       </c>
+      <c r="C25">
+        <f t="shared" si="0"/>
+        <v>58.182295944482966</v>
+      </c>
       <c r="D25">
         <v>0.99</v>
       </c>
@@ -2327,10 +2475,14 @@
         <v>5.04</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26">
         <v>9.76</v>
       </c>
+      <c r="C26">
+        <f t="shared" si="0"/>
+        <v>61.323888598072763</v>
+      </c>
       <c r="D26">
         <v>0.78</v>
       </c>
@@ -2341,9 +2493,13 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27">
         <v>10.27</v>
+      </c>
+      <c r="C27">
+        <f t="shared" si="0"/>
+        <v>64.528313104734352</v>
       </c>
       <c r="D27">
         <v>0.62</v>

</xml_diff>